<commit_message>
Verified rule and added test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000779/negative/01/data/unit-test-coreid-CG0376-negative.xlsx
+++ b/rules/CORE-000779/negative/01/data/unit-test-coreid-CG0376-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000779\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9034DD3-77B5-4220-ADD2-AC96165DE4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9CB988B-8D17-4A36-A930-1BEFEB990C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31440" yWindow="2640" windowWidth="21600" windowHeight="11235" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
   <si>
     <t>Product</t>
   </si>
@@ -143,6 +143,15 @@
   </si>
   <si>
     <t>Record</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>P1.5D</t>
+  </si>
+  <si>
+    <t>p1d</t>
   </si>
 </sst>
 </file>
@@ -215,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -229,6 +238,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -585,7 +597,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -646,6 +658,66 @@
       </c>
       <c r="F3" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -655,7 +727,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -812,6 +884,48 @@
         <v>38</v>
       </c>
     </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adjusted based on PR feedback
</commit_message>
<xml_diff>
--- a/rules/CORE-000779/negative/01/data/unit-test-coreid-CG0376-negative.xlsx
+++ b/rules/CORE-000779/negative/01/data/unit-test-coreid-CG0376-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000779\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9CB988B-8D17-4A36-A930-1BEFEB990C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C80BD16-4B04-40E4-8058-5C1345FC73CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31440" yWindow="2640" windowWidth="21600" windowHeight="11235" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4695" yWindow="2415" windowWidth="21600" windowHeight="11235" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -597,7 +597,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -719,6 +719,9 @@
       <c r="F6" s="7" t="s">
         <v>42</v>
       </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F7" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>